<commit_message>
Paiements exécutés : diminuent les prévisions, pas les soldes bancaires
Plus aucune déduction sur le compte débité ; un reporting où des paiements
avaient été déduits est rétabli à la réimportation. Corrige la relecture
des entités dans un reporting non recalculé par Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NEhkcxCB327Mdpf33KqYQU
</commit_message>
<xml_diff>
--- a/Controle_Reporting_CIV_30-09-2026.xlsx
+++ b/Controle_Reporting_CIV_30-09-2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="265">
   <si>
     <t>Position de trésorerie CI – soldes bancaires au 30/09/2026</t>
   </si>
@@ -368,7 +368,7 @@
     <t>Total comptes de sociétés + comptes dédiés</t>
   </si>
   <si>
-    <t>Comptes indisponibles exclus. Écart = soldes mis à jour et paiements exécutés déduits depuis la position.</t>
+    <t>Comptes indisponibles exclus. Écart = soldes mis à jour à la main depuis la position.</t>
   </si>
   <si>
     <t>2. Fonctionnement : reporting vs RECAP de l'audit (S1 à S4 de l'audit, M FCFA)</t>
@@ -446,7 +446,7 @@
     <t>SCO AO : 15 ligne(s) du reporting modifié remplacées par la prévision de trésorerie SCO.</t>
   </si>
   <si>
-    <t>Paiements exécutés : 4 paiement(s), 704,7 M ; 704,7 M imputés sur le besoin S1 à S5, déduits du solde des comptes débités.</t>
+    <t>Paiements exécutés : 4 paiement(s), 704,7 M ; 704,7 M imputés sur les prévisions S1 à S5 (soldes bancaires inchangés).</t>
   </si>
   <si>
     <t>Comparaison avec la présentation RCI (Laureen) – mêmes sources, M FCFA</t>
@@ -479,9 +479,6 @@
     <t>Explication</t>
   </si>
   <si>
-    <t>Même besoin · Trésorerie : -704,7 (comptes « Dédié paiement Projet SCO » ou comptes non classés en fonctionnement)</t>
-  </si>
-  <si>
     <t>Même besoin</t>
   </si>
   <si>
@@ -596,7 +593,7 @@
     <t>Paiements exécutés depuis la position – diminution des besoins</t>
   </si>
   <si>
-    <t>Montant imputé : déduit du reste à payer des lignes indiquées (feuilles de détail, colonnes « Payé »). Déduit du solde = O : montant retiré du solde du compte débité dans le reporting.</t>
+    <t>Montant imputé : déduit du reste à payer des lignes indiquées (feuilles de détail, colonnes « Payé »). Les paiements exécutés diminuent uniquement les prévisions : les soldes bancaires ne sont pas modifiés.</t>
   </si>
   <si>
     <t>Réf.</t>
@@ -650,7 +647,7 @@
     <t>S1 19,3 M</t>
   </si>
   <si>
-    <t>O</t>
+    <t>N</t>
   </si>
   <si>
     <t>PX|ECOBANK-PICI|TGCC|07/10/2026|629862023|1</t>
@@ -746,7 +743,7 @@
     <t>Paiements exécutés</t>
   </si>
   <si>
-    <t>2d40a539-PAIEMENTS_EXECUTES.xlsx – chaque paiement est imputé sur les lignes de besoin du bénéficiaire (nom, sinon nature de l'audit PICI Projets), des plus anciennes aux plus récentes ; montant retiré du solde du compte débité s'il est postérieur à la position. Détail dans la feuille « Paiements exécutés » du fichier de contrôle.</t>
+    <t>2d40a539-PAIEMENTS_EXECUTES.xlsx – chaque paiement est imputé sur les lignes de besoin du bénéficiaire (nom, sinon nature de l'audit PICI Projets), des plus anciennes aux plus récentes ; ils diminuent les prévisions, pas les soldes bancaires. Détail dans la feuille « Paiements exécutés » du fichier de contrôle.</t>
   </si>
   <si>
     <t>Comptes indisponibles</t>
@@ -1433,7 +1430,7 @@
         <v>17</v>
       </c>
       <c r="F7" s="5">
-        <v>-336430487</v>
+        <v>368235073</v>
       </c>
       <c r="G7" s="5">
         <f>F7/655.957</f>
@@ -2490,7 +2487,7 @@
         <v>116</v>
       </c>
       <c r="B5" s="5">
-        <v>6045814152</v>
+        <v>6750479712</v>
       </c>
       <c r="C5" s="5">
         <v>6750479712</v>
@@ -2915,16 +2912,16 @@
         <v>396.566951</v>
       </c>
       <c r="F5" s="16">
-        <v>-308.098609</v>
+        <v>396.566951</v>
       </c>
       <c r="G5" s="16">
         <v>99.98971200000005</v>
       </c>
       <c r="H5" s="16">
-        <v>-604.675848</v>
+        <v>99.98971200000005</v>
       </c>
       <c r="I5" s="16">
-        <v>-704.66556</v>
+        <v>0</v>
       </c>
       <c r="J5" s="17" t="s">
         <v>154</v>
@@ -2959,7 +2956,7 @@
         <v>-5.684341886080802e-14</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -2991,7 +2988,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -3023,7 +3020,7 @@
         <v>1.4210854715202004e-14</v>
       </c>
       <c r="J8" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -3049,7 +3046,7 @@
         <v>-29.545979600000003</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -3081,7 +3078,7 @@
         <v>2.842170943040401e-14</v>
       </c>
       <c r="J10" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -3113,7 +3110,7 @@
         <v>0</v>
       </c>
       <c r="J11" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -3145,7 +3142,7 @@
         <v>-1.4210854715202004e-14</v>
       </c>
       <c r="J12" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -3171,7 +3168,7 @@
         <v>2.75188</v>
       </c>
       <c r="J13" s="17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -3203,7 +3200,7 @@
         <v>-1.7763568394002505e-15</v>
       </c>
       <c r="J14" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -3235,12 +3232,12 @@
         <v>-1.4210854715202004e-14</v>
       </c>
       <c r="J15" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B16" s="19">
         <v>1568.3964222129398</v>
@@ -3255,16 +3252,16 @@
         <v>745.306796</v>
       </c>
       <c r="F16" s="19">
-        <v>72.52454999999998</v>
+        <v>777.19011</v>
       </c>
       <c r="G16" s="19">
         <v>-693.5213609829399</v>
       </c>
       <c r="H16" s="19">
-        <v>-1424.98102058294</v>
+        <v>-720.31546058294</v>
       </c>
       <c r="I16" s="19">
-        <v>-731.4596596000001</v>
+        <v>-26.794099600000045</v>
       </c>
       <c r="J16" s="18" t="s">
         <v>74</v>
@@ -3272,15 +3269,15 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>112</v>
@@ -3294,7 +3291,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B20" s="16">
         <v>244.99626199999997</v>
@@ -3306,12 +3303,12 @@
         <v>0</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B21" s="16">
         <v>637.405803</v>
@@ -3323,12 +3320,12 @@
         <v>0</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B22" s="16">
         <v>152.070689</v>
@@ -3340,12 +3337,12 @@
         <v>0</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B23" s="16">
         <v>85.788691</v>
@@ -3357,12 +3354,12 @@
         <v>0</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B24" s="16">
         <v>448.13497721294</v>
@@ -3374,12 +3371,12 @@
         <v>0</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B25" s="16">
         <v>129.56826523</v>
@@ -3391,12 +3388,12 @@
         <v>-2.842170943040401e-14</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B26" s="16">
         <v>0</v>
@@ -3408,23 +3405,23 @@
         <v>178.0456286</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>173</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>174</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>114</v>
@@ -3447,12 +3444,12 @@
         <v>4.547473508864641e-13</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B31" s="16">
         <v>91.2699500964329</v>
@@ -3464,12 +3461,12 @@
         <v>0</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B32" s="16">
         <v>1976.5850833750312</v>
@@ -3481,12 +3478,12 @@
         <v>0</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B33" s="16">
         <v>1267.9055957833798</v>
@@ -3498,12 +3495,12 @@
         <v>2.2737367544323206e-13</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B34" s="16">
         <v>455.07613148087546</v>
@@ -3515,12 +3512,12 @@
         <v>-1.1368683772161603e-13</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B35" s="16">
         <v>2643.139493</v>
@@ -3532,7 +3529,7 @@
         <v>0</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -3549,12 +3546,12 @@
         <v>-704.6655599999999</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B37" s="16">
         <v>116.22847414168119</v>
@@ -3566,12 +3563,12 @@
         <v>1.4210854715202004e-14</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B38" s="16">
         <v>2197.7624460785723</v>
@@ -3583,12 +3580,12 @@
         <v>0</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B39" s="16">
         <v>490.0631747136942</v>
@@ -3600,12 +3597,12 @@
         <v>0</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B40" s="16">
         <v>1238.4883764116369</v>
@@ -3617,12 +3614,12 @@
         <v>-2.2737367544323206e-13</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B41" s="16">
         <v>1481.90449</v>
@@ -3634,17 +3631,17 @@
         <v>0</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="20" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B44" s="20"/>
       <c r="C44" s="20"/>
@@ -3658,7 +3655,7 @@
     </row>
     <row r="45" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="20" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B45" s="20"/>
       <c r="C45" s="20"/>
@@ -3672,7 +3669,7 @@
     </row>
     <row r="46" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B46" s="20"/>
       <c r="C46" s="20"/>
@@ -3686,7 +3683,7 @@
     </row>
     <row r="47" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B47" s="20"/>
       <c r="C47" s="20"/>
@@ -3700,7 +3697,7 @@
     </row>
     <row r="48" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="20" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B48" s="20"/>
       <c r="C48" s="20"/>
@@ -3714,7 +3711,7 @@
     </row>
     <row r="49" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="20" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B49" s="20"/>
       <c r="C49" s="20"/>
@@ -3728,7 +3725,7 @@
     </row>
     <row r="50" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="20" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B50" s="20"/>
       <c r="C50" s="20"/>
@@ -3776,67 +3773,67 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>197</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>198</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>203</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>205</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>206</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>207</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>208</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>31</v>
@@ -3845,10 +3842,10 @@
         <v>19324742</v>
       </c>
       <c r="H5" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>209</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>210</v>
       </c>
       <c r="J5" s="5">
         <v>19324742</v>
@@ -3857,24 +3854,24 @@
         <v>0</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>207</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>208</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>31</v>
@@ -3883,10 +3880,10 @@
         <v>629862023</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="J6" s="5">
         <v>629862023</v>
@@ -3895,24 +3892,24 @@
         <v>0</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>207</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>208</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>31</v>
@@ -3921,10 +3918,10 @@
         <v>52769692</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J7" s="5">
         <v>52769692</v>
@@ -3933,24 +3930,24 @@
         <v>0</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>31</v>
@@ -3959,10 +3956,10 @@
         <v>2709103</v>
       </c>
       <c r="H8" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>218</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>219</v>
       </c>
       <c r="J8" s="5">
         <v>2709103</v>
@@ -3971,12 +3968,12 @@
         <v>0</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="6:11" x14ac:dyDescent="0.25">
       <c r="F9" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G9" s="21">
         <f>SUM(G5:G8)</f>
@@ -4005,45 +4002,45 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B3" s="23"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
+        <v>221</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>222</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
+        <v>223</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>224</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
+        <v>225</v>
+      </c>
+      <c r="B6" s="20" t="s">
         <v>226</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="24" t="s">
+        <v>227</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>228</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -4051,15 +4048,15 @@
         <v>45</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
+        <v>230</v>
+      </c>
+      <c r="B9" s="20" t="s">
         <v>231</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -4072,80 +4069,80 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B11" s="23"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="24" t="s">
+        <v>233</v>
+      </c>
+      <c r="B12" s="20" t="s">
         <v>234</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
+        <v>235</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>236</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
+        <v>238</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>239</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
+        <v>241</v>
+      </c>
+      <c r="B17" s="20" t="s">
         <v>242</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="24" t="s">
+        <v>243</v>
+      </c>
+      <c r="B18" s="20" t="s">
         <v>244</v>
-      </c>
-      <c r="B18" s="20" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
+        <v>245</v>
+      </c>
+      <c r="B19" s="20" t="s">
         <v>246</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
+        <v>247</v>
+      </c>
+      <c r="B20" s="20" t="s">
         <v>248</v>
-      </c>
-      <c r="B20" s="20" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -4158,32 +4155,32 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="22" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B22" s="23"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="24" t="s">
+        <v>250</v>
+      </c>
+      <c r="B23" s="20" t="s">
         <v>251</v>
-      </c>
-      <c r="B23" s="20" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="s">
+        <v>252</v>
+      </c>
+      <c r="B24" s="20" t="s">
         <v>253</v>
-      </c>
-      <c r="B24" s="20" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
+        <v>254</v>
+      </c>
+      <c r="B25" s="20" t="s">
         <v>255</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -4196,40 +4193,40 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="22" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B27" s="23"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="24" t="s">
+        <v>257</v>
+      </c>
+      <c r="B28" s="20" t="s">
         <v>258</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="24" t="s">
+        <v>259</v>
+      </c>
+      <c r="B29" s="20" t="s">
         <v>260</v>
-      </c>
-      <c r="B29" s="20" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="24" t="s">
+        <v>261</v>
+      </c>
+      <c r="B30" s="20" t="s">
         <v>262</v>
-      </c>
-      <c r="B30" s="20" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="24" t="s">
+        <v>263</v>
+      </c>
+      <c r="B31" s="20" t="s">
         <v>264</v>
-      </c>
-      <c r="B31" s="20" t="s">
-        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remet la feuille « Paiements exécutés » dans le reporting
Les autres feuilles de contrôle restent dans le fichier de contrôle séparé.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NEhkcxCB327Mdpf33KqYQU
</commit_message>
<xml_diff>
--- a/Controle_Reporting_CIV_30-09-2026.xlsx
+++ b/Controle_Reporting_CIV_30-09-2026.xlsx
@@ -7,15 +7,14 @@
     <sheet sheetId="1" name="Position CI 30-09" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Contrôles" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Comparaison RCI" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Paiements exécutés" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Méthode &amp; sources" state="visible" r:id="rId8"/>
+    <sheet sheetId="4" name="Méthode &amp; sources" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="237">
   <si>
     <t>Position de trésorerie CI – soldes bancaires au 30/09/2026</t>
   </si>
@@ -590,90 +589,6 @@
     <t>• Comptes indisponibles exclus de la position du reporting : STANBIC-FIRST _ Debt Service, STANBIC-FIRST_LL, STANBIC-FIRST_Disbursement, BNI-RIVIERA(Augmentation), BNI-RIVIERA(DSRA) / Placement (1 195,6 M). La présentation RCI exclut aussi ces fonds (DSR, augmentation, LL, disbursement).</t>
   </si>
   <si>
-    <t>Paiements exécutés depuis la position – diminution des besoins</t>
-  </si>
-  <si>
-    <t>Montant imputé : déduit du reste à payer des lignes indiquées (feuilles de détail, colonnes « Payé »). Les paiements exécutés diminuent uniquement les prévisions : les soldes bancaires ne sont pas modifiés.</t>
-  </si>
-  <si>
-    <t>Réf.</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Compte débité</t>
-  </si>
-  <si>
-    <t>Bénéficiaire</t>
-  </si>
-  <si>
-    <t>Projet</t>
-  </si>
-  <si>
-    <t>Montant payé FCFA</t>
-  </si>
-  <si>
-    <t>Imputé sur</t>
-  </si>
-  <si>
-    <t>Répartition</t>
-  </si>
-  <si>
-    <t>Imputé S1 à S5 FCFA</t>
-  </si>
-  <si>
-    <t>Non imputé / hors horizon FCFA</t>
-  </si>
-  <si>
-    <t>Déduit du solde</t>
-  </si>
-  <si>
-    <t>PX|ECOBANK-PICI|TGCC|07/10/2026|19324742|0</t>
-  </si>
-  <si>
-    <t>07/10/2026</t>
-  </si>
-  <si>
-    <t>TGCC</t>
-  </si>
-  <si>
-    <t>NOTRE PÈRE</t>
-  </si>
-  <si>
-    <t>BCC 0017 02 GROS ŒUVRE &amp; INSTALLATION DE CHANTIER</t>
-  </si>
-  <si>
-    <t>S1 19,3 M</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>PX|ECOBANK-PICI|TGCC|07/10/2026|629862023|1</t>
-  </si>
-  <si>
-    <t>S1 373,4 M ; S2 256,5 M</t>
-  </si>
-  <si>
-    <t>PX|ECOBANK-PICI|TGCC|07/10/2026|52769692|2</t>
-  </si>
-  <si>
-    <t>S2 52,8 M</t>
-  </si>
-  <si>
-    <t>PX|ECOBANK-PICI|HORECAF|07/10/2026|2709103|3</t>
-  </si>
-  <si>
-    <t>HORECAF</t>
-  </si>
-  <si>
-    <t>HON 0002 BET / MOE / SSI – SCO</t>
-  </si>
-  <si>
-    <t>S1 2,7 M</t>
-  </si>
-  <si>
     <t>Méthode, règles de semaine et sources</t>
   </si>
   <si>
@@ -743,7 +658,7 @@
     <t>Paiements exécutés</t>
   </si>
   <si>
-    <t>2d40a539-PAIEMENTS_EXECUTES.xlsx – chaque paiement est imputé sur les lignes de besoin du bénéficiaire (nom, sinon nature de l'audit PICI Projets), des plus anciennes aux plus récentes ; ils diminuent les prévisions, pas les soldes bancaires. Détail dans la feuille « Paiements exécutés » du fichier de contrôle.</t>
+    <t>2d40a539-PAIEMENTS_EXECUTES.xlsx – chaque paiement est imputé sur les lignes de besoin du bénéficiaire (nom, sinon nature de l'audit PICI Projets), des plus anciennes aux plus récentes ; ils diminuent les prévisions, pas les soldes bancaires. Détail dans la feuille « Paiements exécutés » du reporting et dans la colonne « Paiement exécuté » des feuilles de détail.</t>
   </si>
   <si>
     <t>Comptes indisponibles</t>
@@ -911,7 +826,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -939,7 +854,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3754,245 +3668,6 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="44" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="10" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="5">
-        <v>19324742</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="J5" s="5">
-        <v>19324742</v>
-      </c>
-      <c r="K5" s="5">
-        <v>0</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="5">
-        <v>629862023</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="J6" s="5">
-        <v>629862023</v>
-      </c>
-      <c r="K6" s="5">
-        <v>0</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="5">
-        <v>52769692</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="J7" s="5">
-        <v>52769692</v>
-      </c>
-      <c r="K7" s="5">
-        <v>0</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="5">
-        <v>2709103</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="J8" s="5">
-        <v>2709103</v>
-      </c>
-      <c r="K8" s="5">
-        <v>0</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="9" spans="6:11" x14ac:dyDescent="0.25">
-      <c r="F9" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="G9" s="21">
-        <f>SUM(G5:G8)</f>
-      </c>
-      <c r="J9" s="21">
-        <f>SUM(J5:J8)</f>
-      </c>
-      <c r="K9" s="21">
-        <f>SUM(K5:K8)</f>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -4002,65 +3677,65 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>219</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="B3" s="23"/>
+      <c r="A3" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="B3" s="22"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="24" t="s">
-        <v>221</v>
+      <c r="A4" s="23" t="s">
+        <v>193</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>222</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
-        <v>223</v>
+      <c r="A5" s="23" t="s">
+        <v>195</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>224</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
-        <v>225</v>
+      <c r="A6" s="23" t="s">
+        <v>197</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>226</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="24" t="s">
-        <v>227</v>
+      <c r="A7" s="23" t="s">
+        <v>199</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>228</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="23" t="s">
         <v>45</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>229</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="24" t="s">
-        <v>230</v>
+      <c r="A9" s="23" t="s">
+        <v>202</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>231</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="23" t="s">
         <v>74</v>
       </c>
       <c r="B10" s="20" t="s">
@@ -4068,85 +3743,85 @@
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
-        <v>232</v>
-      </c>
-      <c r="B11" s="23"/>
+      <c r="A11" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="B11" s="22"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="24" t="s">
-        <v>233</v>
+      <c r="A12" s="23" t="s">
+        <v>205</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>234</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="24" t="s">
-        <v>235</v>
+      <c r="A13" s="23" t="s">
+        <v>207</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>236</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="24" t="s">
-        <v>227</v>
+      <c r="A14" s="23" t="s">
+        <v>199</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>237</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="24" t="s">
-        <v>238</v>
+      <c r="A15" s="23" t="s">
+        <v>210</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="24" t="s">
-        <v>230</v>
+      <c r="A16" s="23" t="s">
+        <v>202</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>240</v>
+        <v>212</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="24" t="s">
-        <v>241</v>
+      <c r="A17" s="23" t="s">
+        <v>213</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>242</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="24" t="s">
-        <v>243</v>
+      <c r="A18" s="23" t="s">
+        <v>215</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>244</v>
+        <v>216</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
-        <v>245</v>
+      <c r="A19" s="23" t="s">
+        <v>217</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>246</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="24" t="s">
-        <v>247</v>
+      <c r="A20" s="23" t="s">
+        <v>219</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>248</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="23" t="s">
         <v>74</v>
       </c>
       <c r="B21" s="20" t="s">
@@ -4154,37 +3829,37 @@
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="B22" s="23"/>
+      <c r="A22" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="B22" s="22"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="24" t="s">
-        <v>250</v>
+      <c r="A23" s="23" t="s">
+        <v>222</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>251</v>
+        <v>223</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="24" t="s">
-        <v>252</v>
+      <c r="A24" s="23" t="s">
+        <v>224</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>253</v>
+        <v>225</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="24" t="s">
-        <v>254</v>
+      <c r="A25" s="23" t="s">
+        <v>226</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>255</v>
+        <v>227</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="24" t="s">
+      <c r="A26" s="23" t="s">
         <v>74</v>
       </c>
       <c r="B26" s="20" t="s">
@@ -4192,41 +3867,41 @@
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="22" t="s">
-        <v>256</v>
-      </c>
-      <c r="B27" s="23"/>
+      <c r="A27" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="B27" s="22"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
-        <v>257</v>
+      <c r="A28" s="23" t="s">
+        <v>229</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>258</v>
+        <v>230</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="24" t="s">
-        <v>259</v>
+      <c r="A29" s="23" t="s">
+        <v>231</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>260</v>
+        <v>232</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="24" t="s">
-        <v>261</v>
+      <c r="A30" s="23" t="s">
+        <v>233</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>262</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="24" t="s">
-        <v>263</v>
+      <c r="A31" s="23" t="s">
+        <v>235</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>264</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>